<commit_message>
Version final todo funcional al 100%
</commit_message>
<xml_diff>
--- a/public/templates/desprendible.xlsx
+++ b/public/templates/desprendible.xlsx
@@ -20,10 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
-  <si>
-    <t xml:space="preserve">Comprobante de Nómina</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t xml:space="preserve">Periodo de Pago:</t>
   </si>
@@ -60,6 +57,18 @@
   <si>
     <t xml:space="preserve">NETO A PAGAR</t>
   </si>
+  <si>
+    <t xml:space="preserve">Elaborado por:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autorizado por:</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Luna Torres</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Carolina Diaz</t>
+  </si>
 </sst>
 </file>
 
@@ -70,7 +79,7 @@
     <numFmt numFmtId="165" formatCode="[$$-240A]#,##0.00;[RED]\-[$$-240A]#,##0.00"/>
     <numFmt numFmtId="166" formatCode="&quot;$ &quot;#,##0;[RED]&quot;-$ &quot;#,##0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -118,6 +127,22 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Bookman Old Style"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <u val="single"/>
       <sz val="11"/>
       <color theme="1"/>
@@ -140,7 +165,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -169,6 +194,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -195,7 +234,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -268,7 +307,23 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -355,9 +410,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>457560</xdr:colOff>
+      <xdr:colOff>456480</xdr:colOff>
       <xdr:row>9</xdr:row>
-      <xdr:rowOff>141840</xdr:rowOff>
+      <xdr:rowOff>140760</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -371,7 +426,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="495360" y="905040"/>
-          <a:ext cx="3113640" cy="951480"/>
+          <a:ext cx="3112560" cy="950400"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -382,6 +437,78 @@
         </a:ln>
       </xdr:spPr>
     </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="twoCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>171360</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>1365120</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>171360</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp>
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="1" name="Conector recto 3"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="4581360"/>
+          <a:ext cx="4516920" cy="360"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="28575">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:miter/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>19800</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>190440</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>2145600</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>190440</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp>
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="2" name="Conector recto 1"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4610880" y="4600440"/>
+          <a:ext cx="4039920" cy="360"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="28575">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:miter/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -564,7 +691,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E1000"/>
+  <dimension ref="A1:F1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.71"/>
@@ -575,9 +702,7 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
+      <c r="A1" s="2"/>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -604,7 +729,7 @@
       <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="4" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="5"/>
     </row>
@@ -612,7 +737,7 @@
       <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="6" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" s="7"/>
     </row>
@@ -620,7 +745,7 @@
       <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="6" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D7" s="7"/>
     </row>
@@ -628,7 +753,7 @@
       <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="6" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D8" s="8"/>
     </row>
@@ -636,7 +761,7 @@
       <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="6" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D9" s="7"/>
       <c r="E9" s="9"/>
@@ -645,32 +770,32 @@
       <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="6" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11" s="11"/>
       <c r="C11" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="11"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D11" s="11"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
+      <c r="B12" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="C12" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="C12" s="12" t="s">
-        <v>11</v>
-      </c>
       <c r="D12" s="12" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -699,19 +824,55 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C18" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="17"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="18"/>
+      <c r="B20" s="18"/>
+      <c r="C20" s="18"/>
+      <c r="D20" s="18"/>
+    </row>
+    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="D18" s="17"/>
-    </row>
-    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B21" s="18"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="20"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18"/>
-    </row>
-    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
-    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+      <c r="A22" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="D22" s="21"/>
+    </row>
+    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="21"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="F23" s="22"/>
+    </row>
+    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="21"/>
+      <c r="B24" s="21"/>
+      <c r="C24" s="21"/>
+      <c r="D24" s="21"/>
+    </row>
+    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="21"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
+      <c r="D25" s="21"/>
+    </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1688,11 +1849,16 @@
     <row r="999" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="1000" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="9">
     <mergeCell ref="A1:D4"/>
     <mergeCell ref="A5:B10"/>
     <mergeCell ref="A11:B11"/>
     <mergeCell ref="C11:D11"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="A22:B25"/>
+    <mergeCell ref="C22:D25"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>